<commit_message>
feat(F-NAR-019): TREE-DIF-041 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-041.xlsx
+++ b/stories/arbres/TREE-DIF-041.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La gare du village sent le café. Les pierres du quai brillent, mouillées. Un train long attend, silencieux. Ça sent le sel, mêlé au café. Une flaque tremble entre deux pierres. Un sac de papier laisse filer de la chaleur. Le pain est tiède, Amir. Les billets sont dans ma poche. Un goéland passe, trop haut pour le quai. La mer est derrière, pas loin. Nina est dans le wagon. Je veux lui montrer la mer. En ce moment, Amir monte la marche. Le marchepied est haut. Merci, tu tiens le sac bien. On va jusqu'à la mer. Le papier du pain craque, chaud.</t>
+          <t>La gare du village sent le café. Les pierres du quai brillent, mouillées. Un train long attend, silencieux. Ça sent le sel, mêlé au café. Une flaque tremble entre deux pierres. Un sac de papier laisse filer de la chaleur. Le pain tiède est à toi, Amir. Les billets sont dans ma poche. Un goéland passe, trop haut pour le quai. La mer est derrière, pas loin. Nina est dans le wagon. Je veux lui montrer la mer. En ce moment, Amir monte la marche. Le marchepied est haut. Merci, tu tiens le sac bien. On va jusqu'à la mer. Le papier du pain craque, chaud.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La gare du village sent le café. Les pierres du quai brillent, mouillées. Un train long attend, silencieux. Ça sent le sel, mêlé au café. Une flaque tremble entre deux pierres. Un sac de papier laisse filer de la chaleur. Le pain est tiède, Amir. Les billets sont dans ma poche. Un goéland passe, trop haut pour le quai. La mer est derrière, pas loin. Nina est dans le wagon. Je veux lui montrer la mer. En ce moment, Amir monte la marche. Le marchepied est haut. Merci, tu tiens le sac bien. On va jusqu'à la mer. Le papier du pain craque, chaud.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La gare du village sent le café. Les pierres du quai brillent, mouillées. Un train long attend, silencieux. Ça sent le sel, mêlé au café. Une flaque tremble entre deux pierres. Un sac de papier laisse filer de la chaleur. Le &lt;emphasis level="moderate"&gt;pain tiède&lt;/emphasis&gt; est à toi, Amir. Les billets sont dans ma poche. Un goéland passe, trop haut pour le quai. La mer est derrière, pas loin. Nina est dans le wagon. Je veux lui montrer la mer. En ce moment, Amir monte la marche. Le marchepied est haut. Merci, tu tiens le sac bien. On va jusqu'à la mer. Le papier du pain craque, chaud.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>La gare du village sent le café. Les pierres du quai brillent, mouillées. Un train long attend, silencieux. Ça sent le sel, mêlé au café. Une flaque tremble entre deux pierres. Un sac de papier laisse filer de la chaleur. Le pain est tiède, Amir. Les billets sont dans ma poche. Un goéland passe, trop haut pour le quai. La mer est derrière, pas loin. Nina est dans le wagon. Je veux lui montrer la mer. En ce moment, Amir monte la marche. Le marchepied est haut. Merci, tu tiens le sac bien. On va jusqu'à la mer. Le papier du pain craque, chaud. [pause]</t>
+          <t>La gare du village sent le café. Les pierres du quai brillent, mouillées. Un train long attend, silencieux. Ça sent le sel, mêlé au café. Une flaque tremble entre deux pierres. Un sac de papier laisse filer de la chaleur. Le &lt;emphasis&gt;pain tiède&lt;/emphasis&gt; est à toi, Amir. Les billets sont dans ma poche. Un goéland passe, trop haut pour le quai. La mer est derrière, pas loin. Nina est dans le wagon. Je veux lui montrer la mer. En ce moment, Amir monte la marche. Le marchepied est haut. Merci, tu tiens le sac bien. On va jusqu'à la mer. Le papier du pain craque, chaud. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1347,7 +1347,7 @@
 narrateur|Ça sent le sel, mêlé au café.
 narrateur|Une flaque tremble entre deux pierres.
 narrateur|Un sac de papier laisse filer de la chaleur.
-maman|Le pain est tiède, Amir.
+maman|Le pain tiède est à toi, Amir.
 papa|Les billets sont dans ma poche.
 narrateur|Un goéland passe, trop haut pour le quai.
 enfant-m|La mer est derrière, pas loin.
@@ -6487,17 +6487,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>On regarde plus tard, alors ? Oui, plus tard. D'accord. La vitre garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir laisse un siège vide, à dessein.</t>
+          <t>On regarde plus tard, alors ? Oui, plus tard. D'accord. La vitre garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir laisse un siège vide, à dessein.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On regarde &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La vitre garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir laisse un siège vide, à dessein.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On regarde &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La vitre garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir laisse un siège vide, à dessein.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>On regarde &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La vitre garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir laisse un siège vide, à dessein. [pause]</t>
+          <t>On regarde &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La vitre garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir laisse un siège vide, à dessein. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6635,7 +6635,7 @@
 enfant-f|Oui, plus tard.
 enfant-m|D'accord.
 narrateur|La vitre garde sa place, sans lui.
-narrateur|Nina serre l'oreille, toujours.
+narrateur|Nina serre l'oreille, sans bouger.
 enfant-f|Garde la mer pour moi.
 enfant-m|Elle t'attend.
 papa|Tu as proposé une autre heure.
@@ -11756,17 +11756,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>On regarde plus tard, alors ? Oui, plus tard. D'accord. La tablette garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Le pain attend, plié, pour deux.</t>
+          <t>On regarde plus tard, alors ? Oui, plus tard. D'accord. La tablette garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Le pain attend, plié, pour deux.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On regarde &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La tablette garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Le pain attend, plié, pour deux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On regarde &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La tablette garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Le pain attend, plié, pour deux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>On regarde &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La tablette garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Le pain attend, plié, pour deux. [pause]</t>
+          <t>On regarde &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La tablette garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Le pain attend, plié, pour deux. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11904,7 +11904,7 @@
 enfant-f|Oui, plus tard.
 enfant-m|D'accord.
 narrateur|La tablette garde sa place, sans lui.
-narrateur|Nina serre l'oreille, toujours.
+narrateur|Nina serre l'oreille, sans bouger.
 enfant-f|Garde la mer pour moi.
 enfant-m|Elle t'attend.
 papa|Tu as proposé une autre heure.
@@ -17022,17 +17022,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>On regarde plus tard, alors ? Oui, plus tard. D'accord. La porte garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir garde un bout de barre, libre.</t>
+          <t>On regarde plus tard, alors ? Oui, plus tard. D'accord. La porte garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir garde un bout de barre, libre.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On regarde &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La porte garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir garde un bout de barre, libre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On regarde &lt;emphasis level="moderate"&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La porte garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir garde un bout de barre, libre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>On regarde &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La porte garde sa place, sans lui. Nina serre l'oreille, toujours. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir garde un bout de barre, libre. [pause]</t>
+          <t>On regarde &lt;emphasis&gt;plus tard&lt;/emphasis&gt;, alors ? Oui, plus tard. D'accord. La porte garde sa place, sans lui. Nina serre l'oreille, sans bouger. Garde la mer pour moi. Elle t'attend. Tu as proposé une autre heure. Elle a dit oui, pour plus tard. Amir garde un bout de barre, libre. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17170,7 +17170,7 @@
 enfant-f|Oui, plus tard.
 enfant-m|D'accord.
 narrateur|La porte garde sa place, sans lui.
-narrateur|Nina serre l'oreille, toujours.
+narrateur|Nina serre l'oreille, sans bouger.
 enfant-f|Garde la mer pour moi.
 enfant-m|Elle t'attend.
 papa|Tu as proposé une autre heure.
@@ -17389,7 +17389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17446,6 +17446,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>